<commit_message>
check test cases product done
</commit_message>
<xml_diff>
--- a/docs/OMS_TestCases_BVA_EP_EN.xlsx
+++ b/docs/OMS_TestCases_BVA_EP_EN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\STUDY\SWIN\Lab\JDA\llmagent4code\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30058A12-0915-4A7B-8BD0-23F5600E0EF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FA783E4-FA95-40E6-AD4A-057D7B2B7635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10236" yWindow="0" windowWidth="12900" windowHeight="13776" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14088" yWindow="0" windowWidth="9048" windowHeight="13776" tabRatio="500" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -3051,7 +3051,7 @@
       <c r="L7" s="16"/>
       <c r="M7" s="16"/>
     </row>
-    <row r="8" spans="1:13" ht="79.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="66" x14ac:dyDescent="0.3">
       <c r="A8" s="16" t="s">
         <v>92</v>
       </c>
@@ -3419,7 +3419,7 @@
       <c r="L17" s="16"/>
       <c r="M17" s="16"/>
     </row>
-    <row r="18" spans="1:13" s="18" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" s="18" customFormat="1" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A18" s="16" t="s">
         <v>135</v>
       </c>
@@ -3456,7 +3456,7 @@
       <c r="L18" s="16"/>
       <c r="M18" s="16"/>
     </row>
-    <row r="19" spans="1:13" s="15" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" s="15" customFormat="1" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A19" s="14" t="s">
         <v>138</v>
       </c>
@@ -4850,153 +4850,153 @@
       <c r="L4" s="13"/>
       <c r="M4" s="13"/>
     </row>
-    <row r="5" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:13" s="15" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="14" t="s">
         <v>269</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="14" t="s">
         <v>270</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="14" t="s">
         <v>271</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="14" t="s">
         <v>272</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="14" t="s">
         <v>273</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="14" t="s">
         <v>274</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-    </row>
-    <row r="6" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+    </row>
+    <row r="6" spans="1:13" s="18" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="16" t="s">
         <v>275</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="16" t="s">
         <v>270</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="16" t="s">
         <v>276</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="16" t="s">
         <v>277</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="16" t="s">
         <v>273</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="16" t="s">
         <v>278</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="K6" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-    </row>
-    <row r="7" spans="1:13" ht="330" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+    </row>
+    <row r="7" spans="1:13" s="18" customFormat="1" ht="330" x14ac:dyDescent="0.3">
+      <c r="A7" s="16" t="s">
         <v>279</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="16" t="s">
         <v>270</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="16" t="s">
         <v>280</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="16" t="s">
         <v>281</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="16" t="s">
         <v>273</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="16" t="s">
         <v>278</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="J7" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="K7" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-    </row>
-    <row r="8" spans="1:13" ht="343.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+    </row>
+    <row r="8" spans="1:13" s="15" customFormat="1" ht="343.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="14" t="s">
         <v>282</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="14" t="s">
         <v>270</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="14" t="s">
         <v>283</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="14" t="s">
         <v>284</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="14" t="s">
         <v>273</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="J8" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="K8" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
+      <c r="L8" s="14"/>
+      <c r="M8" s="14"/>
     </row>
     <row r="9" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
@@ -5107,153 +5107,153 @@
       <c r="L11" s="12"/>
       <c r="M11" s="12"/>
     </row>
-    <row r="12" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:13" s="15" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="14" t="s">
         <v>293</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="14" t="s">
         <v>294</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="14" t="s">
         <v>295</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="14" t="s">
         <v>297</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="J12" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="K12" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-    </row>
-    <row r="13" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="K12" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="L12" s="14"/>
+      <c r="M12" s="14"/>
+    </row>
+    <row r="13" spans="1:13" s="18" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="16" t="s">
         <v>298</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="16" t="s">
         <v>293</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="16" t="s">
         <v>299</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="16" t="s">
         <v>300</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="H13" s="16" t="s">
         <v>296</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="I13" s="16" t="s">
         <v>278</v>
       </c>
-      <c r="J13" s="4" t="s">
+      <c r="J13" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="K13" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
-    </row>
-    <row r="14" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
+      <c r="K13" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L13" s="16"/>
+      <c r="M13" s="16"/>
+    </row>
+    <row r="14" spans="1:13" s="18" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="16" t="s">
         <v>301</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="16" t="s">
         <v>293</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="16" t="s">
         <v>302</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="16" t="s">
         <v>303</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="H14" s="16" t="s">
         <v>296</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I14" s="16" t="s">
         <v>278</v>
       </c>
-      <c r="J14" s="4" t="s">
+      <c r="J14" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="K14" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-    </row>
-    <row r="15" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+      <c r="K14" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L14" s="16"/>
+      <c r="M14" s="16"/>
+    </row>
+    <row r="15" spans="1:13" s="15" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="14" t="s">
         <v>304</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="14" t="s">
         <v>293</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="14" t="s">
         <v>305</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="H15" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="I15" s="14" t="s">
         <v>307</v>
       </c>
-      <c r="J15" s="4" t="s">
+      <c r="J15" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="K15" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
+      <c r="K15" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="L15" s="14"/>
+      <c r="M15" s="14"/>
     </row>
     <row r="16" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A16" s="13" t="s">
@@ -5512,42 +5512,42 @@
       <c r="L22" s="12"/>
       <c r="M22" s="12"/>
     </row>
-    <row r="23" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
+    <row r="23" spans="1:13" s="15" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A23" s="14" t="s">
         <v>337</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="14" t="s">
         <v>327</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="14" t="s">
         <v>338</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="14" t="s">
         <v>339</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="G23" s="14" t="s">
         <v>340</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="H23" s="14" t="s">
         <v>330</v>
       </c>
-      <c r="I23" s="4" t="s">
+      <c r="I23" s="14" t="s">
         <v>341</v>
       </c>
-      <c r="J23" s="4" t="s">
+      <c r="J23" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="K23" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="L23" s="4"/>
-      <c r="M23" s="4"/>
+      <c r="K23" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="L23" s="14"/>
+      <c r="M23" s="14"/>
     </row>
     <row r="24" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A24" s="13" t="s">

</xml_diff>